<commit_message>
scripts: save workbooks atomically via os.replace
</commit_message>
<xml_diff>
--- a/_канон/источники.xlsx
+++ b/_канон/источники.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q28"/>
+  <dimension ref="A1:Q44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2294,6 +2294,1256 @@
       <c r="Q28" t="inlineStr">
         <is>
           <t>ПОИСК_09_Multiproject_Scheduling</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>wwc_wellbeing</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>What Works Centre for Wellbeing</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>What Works Centre for Wellbeing|What Works Wellbeing|WWC Wellbeing</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>whatworkswellbeing.org</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>институция с редакцией</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>университет или институт</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Независимый исследовательский центр, созданный при поддержке Economic and Social Research Council (ESRC), публикует систематические обзоры с описанной методологией</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>https://whatworkswellbeing.org/about-us/</t>
+        </is>
+      </c>
+      <c r="K29" t="n">
+        <v>1</v>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>подтверждено</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>2025-01-28</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Центр работал 2014-2022, специализировался на систематических обзорах доказательств благополучия. Методология описана (GRADE), но без внешнего рецензирования — институциональная ответственность без процедурной проверки</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>scimagojr.com — не журнал; whatworkswellbeing.org — официальный сайт с описанием деятельности; ESRC — подтверждение институциональной принадлежности</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Забота и поддержка_01_work_wellbeing_playbook_a_systematic_review_of_evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>cmhaa</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Corporate Mental Health Alliance Australia</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Corporate Mental Health Alliance Australia|CMHAA</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>cmhaa.org.au</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>институция с редакцией</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>корпоративный или консалтинговый источник</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>официальный домен cmhaa.org.au, индустриальная коалиция работодателей и провайдеров услуг</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>https://cmhaa.org.au</t>
+        </is>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>подтверждено</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>2025-01-17</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Индустриальная ассоциация, выпускающая отчёты о практиках психического здоровья на рабочих местах. Организация идентифицируема, домен официальный, но процедуры независимого рецензирования отчётов нет.</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>cmhaa.org.au; ansi.org accredited developers; scimagojr.com</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Забота и поддержка_03_the_leading_mentally_healthy_workplaces_survey_report_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>us_army_phc</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>U.S. Army Public Health Center</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>U.S. Army Public Health Center|US Army Public Health Center|Army Public Health Center|APHC</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>phc.amedd.army.mil</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>документ ведомства</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>орган власти</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Официальное подразделение U.S. Army Medical Department, публикует на зарезервированном военном домене .mil</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>https://phc.amedd.army.mil/Pages/default.aspx</t>
+        </is>
+      </c>
+      <c r="K31" t="n">
+        <v>2</v>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>подтверждено</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>2025-06-10</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Домен .mil зарезервирован для Министерства обороны США. APHC — официальный центр общественного здравоохранения армии, отвечающий за исследования и рекомендации по охране здоровья военнослужащих</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>phc.amedd.army.mil; U.S. Army Public Health Center official status; .mil domain registry</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>Забота и поддержка_01_supportive_leadership_training_to_improve_social_connec</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>bmj_open_quality</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>BMJ Open Quality</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>BMJ Open Quality|BMJOQ</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>2399-6641</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>bmjopenquality.bmj.com</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>рецензирование</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>научный журнал</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Scimago: Q3 в 2 из 4 категорий (Health Policy Q2, Leadership Q2, Public Health Q3, Strategy Q3), при равенстве берётся худшая</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>scimagojr.com</t>
+        </is>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>подтверждено</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>2025-06-14</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>SJR 0.531 (2023), H-index 28. Журнал BMJ Publishing Group, рецензируемый. Квартиль определён по правилу: Q2 в двух категориях, Q3 в двух — равенство, берётся худший.</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>scimagojr.com по ISSN 2399-6641; portal.issn.org для подтверждения ISSN; bmjopenquality.bmj.com для проверки официального домена</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Забота и поддержка_04_changing_minds_saving_lives_how_training_psychological</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>ais</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Association for Information Systems</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>AIS|Association for Information Systems</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>aisnet.org</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>рецензирование конференции</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>сборник конференции</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Сборники конференций AIS индексируются в Scimago (ICIS, AMCIS, ECIS proceedings), категория без квартилей</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>https://www.scimagojr.com/journalsearch.php?q=association+for+information+systems</t>
+        </is>
+      </c>
+      <c r="K33" t="n">
+        <v>1</v>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>подтверждено</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>2025-06-11</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>AIS организует ведущие конференции по информационным системам. Сборники проходят программный комитет и рецензирование, публикуются в AIS Electronic Library. Scimago индексирует proceedings, но квартилей не присваивает — по правилу строки 2 это +1</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>scimagojr.com: Association for Information Systems; scimagojr.com: ICIS proceedings; aisnet.org: подтверждение организации; portal.issn.org: поиск ISSN для AIS conference proceedings</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Использование технологий для развития продуктов и сервисов_03_optimizing_service_experience_design_with_generative_ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>laurea_uas</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Laurea University of Applied Sciences</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Laurea UAS|Laurea-ammattikorkeakoulu|Laurea</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>laurea.fi</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>институция с редакцией</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>университет или институт</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Аккредитованное высшее учебное заведение в реестре Finnish National Agency for Education</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>https://opintopolku.fi/konfo/en/oppilaitokset, https://www.laurea.fi</t>
+        </is>
+      </c>
+      <c r="K34" t="n">
+        <v>1</v>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>подтверждено</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>2025-01-24</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Финский университет прикладных наук. Публикует через репозиторий Theseus, но без формального внешнего рецензирования. Институциональная ответственность есть, процедура рецензирования отсутствует — поэтому +1, а не +2</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>scimagojr.com: Laurea University; opintopolku.fi: Finnish higher education institutions; isbn-international.org: Laurea; theseus.fi: проверка типа публикаций</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Осознанность в развитии — личный фокус_03_knowledge_workers_self_directed_learning_framework_for</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>sage_open</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>SAGE Open</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>SAGE Open|Sage Open</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>2158-2440</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>sagepub.com</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>рецензирование</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>научный журнал</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Scimago Journal Rank: Q2 во всех категориях (Social Sciences (miscellaneous): Q2, Arts and Humanities (miscellaneous): Q2)</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>https://www.scimagojr.com/journalsearch.php?q=21100200831</t>
+        </is>
+      </c>
+      <c r="K35" t="n">
+        <v>1</v>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>подтверждено</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>2025-06-12</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Open access журнал SAGE Publications. SJR 2023: 0.436, H-index: 90. Междисциплинарный журнал, стабильно Q2 в обеих категориях.</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>Scimago Journal &amp; Country Rank (scimagojr.com); ISSN Portal (portal.issn.org); DOI resolution (doi.org)</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Построение отношений_01_06_the_impact_of_recognition_fairness_and_leadership_on_em</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>bmc_nursing</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>BMC Nursing</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>BMC Nursing|BioMed Central Nursing</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>1472-6955</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>biomedcentral.com</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>рецензирование</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>научный журнал</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Scimago 2023: Q2 в категории Nursing (84-й перцентиль)</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>https://www.scimagojr.com/journalsearch.php?q=19700182406</t>
+        </is>
+      </c>
+      <c r="K36" t="n">
+        <v>1</v>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>подтверждено</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>2025-06-13</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>SJR 0.593, H-index 40. Единственная категория журнала — Nursing Q2, других категорий нет. Издатель BioMed Central (Springer Nature), но строка заводится на конкретный журнал, а не издательство</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>scimagojr.com: BMC Nursing; portal.issn.org: 1472-6955; doi.org: проверка префикса 10.1186</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>Развитие эффективности команды_07_360_Feedback_Development</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>jscimedcentral</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>SciMed Central (Journal of Scientific Medicine)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>SciMed Central|JSciMed Central|Central</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>2333-7125</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>jscimedcentral.com</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Издательство включено в список хищнических издательств Beall's List и Cabells Predatory Reports; отсутствует в Scimago, DOAJ и других авторитетных индексах; отсутствует прозрачная информация о процессе рецензирования</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>beallslist.net, scimagojr.com, doaj.org, jscimedcentral.com</t>
+        </is>
+      </c>
+      <c r="K37" t="n">
+        <v>-2</v>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>подтверждено</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>2025-01-18</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Predatory publisher. Имитация научного журнала: есть ISSN, формальная структура сайта, но нет проверяемого процесса рецензирования, редколлегии, индексирования. Модель pay-to-publish без контроля качества. Невозможно установить ответственность за содержание.</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>Scimago по ISSN 2333-7125; DOAJ по названию и ISSN; Beall's List predatory publishers; Cabells Predatory Reports; официальный сайт jscimedcentral.com</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Развитие эффективности команды_06_teamwork_coaching_in_the_research_development_process</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>heliyon_elsevier</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Heliyon</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Heliyon|Elsevier Heliyon</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>2405-8440</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>elsevier.com</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>рецензирование</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>научный журнал</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Scimago: Q1 в 91 категории из 95</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>https://www.scimagojr.com/journalsearch.php?q=21100814830</t>
+        </is>
+      </c>
+      <c r="K38" t="n">
+        <v>2</v>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>подтверждено</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>2025-01-20</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Междисциплинарный open-access журнал Elsevier. SJR 0.58, H-index 81 (2023). Q1 доминирует в распределении категорий.</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Scimago Journal Rank по ISSN 2405-8440</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>Создание долгосрочной ценности_01_The_impact_of_value_co_creation_behavior_on_customer_loyalty_in_the_s|Создание долгосрочной ценности_01_Customer_experience_management_in_B2B_markets_CXM_value_propositions_</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>gradus_kaposvar</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Gradus</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Gradus|Gradus Journal</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2064-8014</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>gradus.kefo.hu</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>рецензирование</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>научный журнал</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Не найден в Scimago, Scopus, WoS, DOAJ. Журнал зарегистрирован в ISSN Portal, издается Kaposvár University, заявлено peer-review на сайте, но индексации в наукометрических базах нет</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>scimagojr.com, portal.issn.org, doaj.org, gradus.kefo.hu</t>
+        </is>
+      </c>
+      <c r="K39" t="n">
+        <v>1</v>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>ждёт подтверждения</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>2025-01-16</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Университетский журнал без квартиля. Формально заявлен как рецензируемый, но отсутствие в основных базах не позволяет подтвердить процесс. Потолок S = 0 до появления маркера</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Scimago JR по ISSN 2064-8014; ISSN Portal; DOAJ; Scopus coverage; Web of Science Master Journal List</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>Управление конфликтами_01_assessing_the_effectiveness_of_conflict_prevention_and</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>jgme_acgme</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Journal of Graduate Medical Education</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Journal of Graduate Medical Education|JGME|Accreditation Council for Graduate Medical Education</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>1949-8349|1949-8357</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>acgme.org</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>рецензирование</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>научный журнал</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Scimago: Q2 в обеих предметных категориях (Education, Medicine miscellaneous)</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>scimagojr.com/journalsearch.php?q=1949-8357</t>
+        </is>
+      </c>
+      <c r="K40" t="n">
+        <v>1</v>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>подтверждено</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>2025-06-14</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>SJR 0.551, H-index 45. Квартили: Education Q2 (6/268), Medicine (miscellaneous) Q2 (78/363). Издаётся Accreditation Council for Graduate Medical Education, индексируется в PubMed/MEDLINE</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>scimagojr.com по ISSN 1949-8357; portal.issn.org для проверки обоих ISSN</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>Управление конфликтами_02_building_bridges_approaches_to_conflict_resolution_that</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>aj_publishing_ejcm</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>African Journals Publishing, European Journal of Commercial Management</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>AJ Publishing|EJCM|European Journal of Commercial Management</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>2789-7060</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>ajpojournals.org</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>рецензирование</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>научный журнал</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Scimago: не индексируется, DOAJ: не включён, Scopus/WoS: не обнаружен</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>scimagojr.com, portal.issn.org, doaj.org, ajpojournals.org/journals/european-journal-of-commercial-management</t>
+        </is>
+      </c>
+      <c r="K41" t="n">
+        <v>2</v>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>ждёт подтверждения</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>2025-06-12</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>ISSN зарегистрирован, peer review заявлен издателем, но независимого подтверждения качества (индексация в Scimago, DOAJ, Scopus) не найдено. Портфель издательства — несколько open access журналов из Кении, основан недавно (ISSN с 2022). Без маркера S ограничено потолком 0</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Scimago Journal Rank по ISSN 2789-7060; DOAJ по названию и ISSN; SPI (Scientific Publishers Indicator) для AJ Publishing; Scopus/Web of Science coverage через публичные источники; Официальный сайт издательства ajpojournals.org</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Управление конфликтами_04_Mediation_Ghana</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>negotiation_journal</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Negotiation Journal</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Negotiation Journal|Wiley Periodicals, Inc.</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>0748-4526|1571-9979</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>onlinelibrary.wiley.com</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>рецензирование</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>научный журнал</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Scimago: Q2 в Business and International Management, Q2 в Law, Q2 в Management of Technology and Innovation</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>https://www.scimagojr.com/journalsearch.php?q=21619&amp;tip=sid</t>
+        </is>
+      </c>
+      <c r="K42" t="n">
+        <v>1</v>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>подтверждено</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>2025-06-12</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>SJR 0.376, H-index 43. Издаётся Wiley для Program on Negotiation at Harvard Law School. Все три предметные категории — Q2, поэтому S = +1.</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>portal.issn.org для ISSN 0748-4526; scimagojr.com для Negotiation Journal</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>Управление конфликтами_05_Confirming_the_Impact_of_Training_on_Negotiators_and_Organizations</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>univ_florida_ifas</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>University of Florida, Institute of Food and Agricultural Sciences</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>UF/IFAS Extension|University of Florida IFAS|UF IFAS|Университет Флориды IFAS</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>ufl.edu</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>институция с редакцией</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>университет или институт</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>University of Florida имеет региональную аккредитацию SACSCOC (Southern Association of Colleges and Schools Commission on Colleges). Extension публикации — образовательные материалы, не рецензируемые статьи.</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>https://www.ufl.edu/ , https://www.sacscoc.org/</t>
+        </is>
+      </c>
+      <c r="K43" t="n">
+        <v>1</v>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>подтверждено</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>2025-06-12</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>UF/IFAS Extension — служба распространения знаний Университета Флориды. Публикует образовательные материалы для фермеров, землевладельцев и широкой публики. Авторы — сотрудники университета с научными степенями. Формат не исследовательский, поэтому +1, не +2.</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>scimagojr.com (по DOI и домену); ansi.org, iso.org; SACSCOC accreditation database; официальный сайт UF/IFAS</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>Управление конфликтами_07_AEC784_WC445_Rahim_Organizational_Conflict_Inventory</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ahfe_open_access</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>AHFE Open Access</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>AHFE Open Access|AHFE International</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2771-0718</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>ahfe.org</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>рецензирование</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>научный журнал</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Scimago: Q4 в обеих категориях (Engineering miscellaneous, Human Factors and Ergonomics)</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>https://www.scimagojr.com/journalsearch.php?q=21101188117</t>
+        </is>
+      </c>
+      <c r="K44" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>подтверждено</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>2025-01-22</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>SJR 2023: 0.163, H-index: 9. Квартиль Q4 в обеих предметных категориях → S = 0 по правилу Q3–Q4</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>Scimago Journal Rank по домену ahfe.org и DOI-префиксу 10.54941; Portal ISSN для подтверждения ISSN</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>Фокус на главном, долгосрочное планирование_03_team_centric_innovation_the_role_of_objectives_and_key</t>
         </is>
       </c>
     </row>

</xml_diff>